<commit_message>
Translated all scripts and logs to English
</commit_message>
<xml_diff>
--- a/STRICT_REPORT_0552.xlsx
+++ b/STRICT_REPORT_0552.xlsx
@@ -1,15 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="4" rupBuild="14420"/>
   <workbookPr defaultThemeVersion="124226"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\user\Desktop\ilia\MyProject2\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
   <bookViews>
     <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="124519"/>
 </workbook>
 </file>
 
@@ -607,8 +612,8 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -658,6 +663,14 @@
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
@@ -704,7 +717,7 @@
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Cambria"/>
+        <a:latin typeface="Cambria" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -736,9 +749,10 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri"/>
+        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
@@ -770,6 +784,7 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
     <a:fmtScheme name="Office">
@@ -945,11 +960,11 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:H106"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:8">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -975,7 +990,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:8">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>100</v>
       </c>
@@ -1001,7 +1016,7 @@
         <v>163</v>
       </c>
     </row>
-    <row r="3" spans="1:8">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>100</v>
       </c>
@@ -1027,7 +1042,7 @@
         <v>164</v>
       </c>
     </row>
-    <row r="4" spans="1:8">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>100</v>
       </c>
@@ -1053,7 +1068,7 @@
         <v>165</v>
       </c>
     </row>
-    <row r="5" spans="1:8">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>100</v>
       </c>
@@ -1079,7 +1094,7 @@
         <v>166</v>
       </c>
     </row>
-    <row r="6" spans="1:8">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>100</v>
       </c>
@@ -1105,7 +1120,7 @@
         <v>167</v>
       </c>
     </row>
-    <row r="7" spans="1:8">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>100</v>
       </c>
@@ -1131,7 +1146,7 @@
         <v>168</v>
       </c>
     </row>
-    <row r="8" spans="1:8">
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>100</v>
       </c>
@@ -1157,7 +1172,7 @@
         <v>169</v>
       </c>
     </row>
-    <row r="9" spans="1:8">
+    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>100</v>
       </c>
@@ -1183,7 +1198,7 @@
         <v>170</v>
       </c>
     </row>
-    <row r="10" spans="1:8">
+    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>100</v>
       </c>
@@ -1209,7 +1224,7 @@
         <v>171</v>
       </c>
     </row>
-    <row r="11" spans="1:8">
+    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>100</v>
       </c>
@@ -1235,7 +1250,7 @@
         <v>165</v>
       </c>
     </row>
-    <row r="12" spans="1:8">
+    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>100</v>
       </c>
@@ -1261,7 +1276,7 @@
         <v>172</v>
       </c>
     </row>
-    <row r="13" spans="1:8">
+    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>100</v>
       </c>
@@ -1287,7 +1302,7 @@
         <v>170</v>
       </c>
     </row>
-    <row r="14" spans="1:8">
+    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>100</v>
       </c>
@@ -1313,7 +1328,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="15" spans="1:8">
+    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A15">
         <v>100</v>
       </c>
@@ -1339,7 +1354,7 @@
         <v>174</v>
       </c>
     </row>
-    <row r="16" spans="1:8">
+    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A16">
         <v>100</v>
       </c>
@@ -1365,7 +1380,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="17" spans="1:8">
+    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A17">
         <v>100</v>
       </c>
@@ -1391,7 +1406,7 @@
         <v>176</v>
       </c>
     </row>
-    <row r="18" spans="1:8">
+    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A18">
         <v>100</v>
       </c>
@@ -1417,7 +1432,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="19" spans="1:8">
+    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A19">
         <v>100</v>
       </c>
@@ -1443,7 +1458,7 @@
         <v>178</v>
       </c>
     </row>
-    <row r="20" spans="1:8">
+    <row r="20" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A20">
         <v>100</v>
       </c>
@@ -1469,7 +1484,7 @@
         <v>179</v>
       </c>
     </row>
-    <row r="21" spans="1:8">
+    <row r="21" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A21">
         <v>100</v>
       </c>
@@ -1495,7 +1510,7 @@
         <v>180</v>
       </c>
     </row>
-    <row r="22" spans="1:8">
+    <row r="22" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A22">
         <v>100</v>
       </c>
@@ -1521,7 +1536,7 @@
         <v>181</v>
       </c>
     </row>
-    <row r="23" spans="1:8">
+    <row r="23" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A23">
         <v>100</v>
       </c>
@@ -1547,7 +1562,7 @@
         <v>182</v>
       </c>
     </row>
-    <row r="24" spans="1:8">
+    <row r="24" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A24">
         <v>100</v>
       </c>
@@ -1573,7 +1588,7 @@
         <v>174</v>
       </c>
     </row>
-    <row r="25" spans="1:8">
+    <row r="25" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A25">
         <v>100</v>
       </c>
@@ -1599,7 +1614,7 @@
         <v>167</v>
       </c>
     </row>
-    <row r="26" spans="1:8">
+    <row r="26" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A26">
         <v>100</v>
       </c>
@@ -1625,7 +1640,7 @@
         <v>183</v>
       </c>
     </row>
-    <row r="27" spans="1:8">
+    <row r="27" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A27">
         <v>100</v>
       </c>
@@ -1651,7 +1666,7 @@
         <v>184</v>
       </c>
     </row>
-    <row r="28" spans="1:8">
+    <row r="28" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A28">
         <v>98</v>
       </c>
@@ -1677,7 +1692,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="29" spans="1:8">
+    <row r="29" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A29">
         <v>98</v>
       </c>
@@ -1703,7 +1718,7 @@
         <v>166</v>
       </c>
     </row>
-    <row r="30" spans="1:8">
+    <row r="30" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A30">
         <v>97</v>
       </c>
@@ -1729,7 +1744,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="31" spans="1:8">
+    <row r="31" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A31">
         <v>97</v>
       </c>
@@ -1755,7 +1770,7 @@
         <v>166</v>
       </c>
     </row>
-    <row r="32" spans="1:8">
+    <row r="32" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A32">
         <v>97</v>
       </c>
@@ -1781,7 +1796,7 @@
         <v>174</v>
       </c>
     </row>
-    <row r="33" spans="1:8">
+    <row r="33" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A33">
         <v>97</v>
       </c>
@@ -1807,7 +1822,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="34" spans="1:8">
+    <row r="34" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A34">
         <v>97</v>
       </c>
@@ -1833,7 +1848,7 @@
         <v>166</v>
       </c>
     </row>
-    <row r="35" spans="1:8">
+    <row r="35" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A35">
         <v>97</v>
       </c>
@@ -1859,7 +1874,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="36" spans="1:8">
+    <row r="36" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A36">
         <v>97</v>
       </c>
@@ -1885,7 +1900,7 @@
         <v>174</v>
       </c>
     </row>
-    <row r="37" spans="1:8">
+    <row r="37" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A37">
         <v>97</v>
       </c>
@@ -1911,7 +1926,7 @@
         <v>166</v>
       </c>
     </row>
-    <row r="38" spans="1:8">
+    <row r="38" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A38">
         <v>97</v>
       </c>
@@ -1937,7 +1952,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="39" spans="1:8">
+    <row r="39" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A39">
         <v>97</v>
       </c>
@@ -1963,7 +1978,7 @@
         <v>166</v>
       </c>
     </row>
-    <row r="40" spans="1:8">
+    <row r="40" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A40">
         <v>97</v>
       </c>
@@ -1989,7 +2004,7 @@
         <v>166</v>
       </c>
     </row>
-    <row r="41" spans="1:8">
+    <row r="41" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A41">
         <v>97</v>
       </c>
@@ -2015,7 +2030,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="42" spans="1:8">
+    <row r="42" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A42">
         <v>97</v>
       </c>
@@ -2041,7 +2056,7 @@
         <v>174</v>
       </c>
     </row>
-    <row r="43" spans="1:8">
+    <row r="43" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A43">
         <v>97</v>
       </c>
@@ -2067,7 +2082,7 @@
         <v>174</v>
       </c>
     </row>
-    <row r="44" spans="1:8">
+    <row r="44" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A44">
         <v>97</v>
       </c>
@@ -2093,7 +2108,7 @@
         <v>164</v>
       </c>
     </row>
-    <row r="45" spans="1:8">
+    <row r="45" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A45">
         <v>97</v>
       </c>
@@ -2119,7 +2134,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="46" spans="1:8">
+    <row r="46" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A46">
         <v>97</v>
       </c>
@@ -2145,7 +2160,7 @@
         <v>174</v>
       </c>
     </row>
-    <row r="47" spans="1:8">
+    <row r="47" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A47">
         <v>96</v>
       </c>
@@ -2171,7 +2186,7 @@
         <v>171</v>
       </c>
     </row>
-    <row r="48" spans="1:8">
+    <row r="48" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A48">
         <v>96</v>
       </c>
@@ -2197,7 +2212,7 @@
         <v>165</v>
       </c>
     </row>
-    <row r="49" spans="1:8">
+    <row r="49" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A49">
         <v>96</v>
       </c>
@@ -2223,7 +2238,7 @@
         <v>176</v>
       </c>
     </row>
-    <row r="50" spans="1:8">
+    <row r="50" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A50">
         <v>96</v>
       </c>
@@ -2249,7 +2264,7 @@
         <v>170</v>
       </c>
     </row>
-    <row r="51" spans="1:8">
+    <row r="51" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A51">
         <v>96</v>
       </c>
@@ -2275,7 +2290,7 @@
         <v>176</v>
       </c>
     </row>
-    <row r="52" spans="1:8">
+    <row r="52" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A52">
         <v>96</v>
       </c>
@@ -2301,7 +2316,7 @@
         <v>171</v>
       </c>
     </row>
-    <row r="53" spans="1:8">
+    <row r="53" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A53">
         <v>96</v>
       </c>
@@ -2327,7 +2342,7 @@
         <v>167</v>
       </c>
     </row>
-    <row r="54" spans="1:8">
+    <row r="54" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A54">
         <v>96</v>
       </c>
@@ -2353,7 +2368,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="55" spans="1:8">
+    <row r="55" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A55">
         <v>96</v>
       </c>
@@ -2379,7 +2394,7 @@
         <v>170</v>
       </c>
     </row>
-    <row r="56" spans="1:8">
+    <row r="56" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A56">
         <v>96</v>
       </c>
@@ -2405,7 +2420,7 @@
         <v>165</v>
       </c>
     </row>
-    <row r="57" spans="1:8">
+    <row r="57" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A57">
         <v>96</v>
       </c>
@@ -2431,7 +2446,7 @@
         <v>167</v>
       </c>
     </row>
-    <row r="58" spans="1:8">
+    <row r="58" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A58">
         <v>94</v>
       </c>
@@ -2457,7 +2472,7 @@
         <v>183</v>
       </c>
     </row>
-    <row r="59" spans="1:8">
+    <row r="59" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A59">
         <v>94</v>
       </c>
@@ -2483,7 +2498,7 @@
         <v>165</v>
       </c>
     </row>
-    <row r="60" spans="1:8">
+    <row r="60" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A60">
         <v>94</v>
       </c>
@@ -2509,7 +2524,7 @@
         <v>167</v>
       </c>
     </row>
-    <row r="61" spans="1:8">
+    <row r="61" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A61">
         <v>94</v>
       </c>
@@ -2535,7 +2550,7 @@
         <v>170</v>
       </c>
     </row>
-    <row r="62" spans="1:8">
+    <row r="62" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A62">
         <v>94</v>
       </c>
@@ -2561,7 +2576,7 @@
         <v>183</v>
       </c>
     </row>
-    <row r="63" spans="1:8">
+    <row r="63" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A63">
         <v>94</v>
       </c>
@@ -2587,7 +2602,7 @@
         <v>170</v>
       </c>
     </row>
-    <row r="64" spans="1:8">
+    <row r="64" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A64">
         <v>94</v>
       </c>
@@ -2613,7 +2628,7 @@
         <v>165</v>
       </c>
     </row>
-    <row r="65" spans="1:8">
+    <row r="65" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A65">
         <v>94</v>
       </c>
@@ -2639,7 +2654,7 @@
         <v>167</v>
       </c>
     </row>
-    <row r="66" spans="1:8">
+    <row r="66" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A66">
         <v>93</v>
       </c>
@@ -2665,7 +2680,7 @@
         <v>172</v>
       </c>
     </row>
-    <row r="67" spans="1:8">
+    <row r="67" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A67">
         <v>93</v>
       </c>
@@ -2691,7 +2706,7 @@
         <v>185</v>
       </c>
     </row>
-    <row r="68" spans="1:8">
+    <row r="68" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A68">
         <v>93</v>
       </c>
@@ -2717,7 +2732,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="69" spans="1:8">
+    <row r="69" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A69">
         <v>93</v>
       </c>
@@ -2743,7 +2758,7 @@
         <v>186</v>
       </c>
     </row>
-    <row r="70" spans="1:8">
+    <row r="70" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A70">
         <v>93</v>
       </c>
@@ -2769,7 +2784,7 @@
         <v>187</v>
       </c>
     </row>
-    <row r="71" spans="1:8">
+    <row r="71" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A71">
         <v>93</v>
       </c>
@@ -2795,7 +2810,7 @@
         <v>166</v>
       </c>
     </row>
-    <row r="72" spans="1:8">
+    <row r="72" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A72">
         <v>93</v>
       </c>
@@ -2821,7 +2836,7 @@
         <v>181</v>
       </c>
     </row>
-    <row r="73" spans="1:8">
+    <row r="73" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A73">
         <v>93</v>
       </c>
@@ -2847,7 +2862,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="74" spans="1:8">
+    <row r="74" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A74">
         <v>93</v>
       </c>
@@ -2873,7 +2888,7 @@
         <v>174</v>
       </c>
     </row>
-    <row r="75" spans="1:8">
+    <row r="75" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A75">
         <v>92</v>
       </c>
@@ -2899,7 +2914,7 @@
         <v>188</v>
       </c>
     </row>
-    <row r="76" spans="1:8">
+    <row r="76" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A76">
         <v>92</v>
       </c>
@@ -2925,7 +2940,7 @@
         <v>175</v>
       </c>
     </row>
-    <row r="77" spans="1:8">
+    <row r="77" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A77">
         <v>92</v>
       </c>
@@ -2951,7 +2966,7 @@
         <v>166</v>
       </c>
     </row>
-    <row r="78" spans="1:8">
+    <row r="78" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A78">
         <v>92</v>
       </c>
@@ -2977,7 +2992,7 @@
         <v>174</v>
       </c>
     </row>
-    <row r="79" spans="1:8">
+    <row r="79" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A79">
         <v>92</v>
       </c>
@@ -3003,7 +3018,7 @@
         <v>189</v>
       </c>
     </row>
-    <row r="80" spans="1:8">
+    <row r="80" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A80">
         <v>92</v>
       </c>
@@ -3029,7 +3044,7 @@
         <v>187</v>
       </c>
     </row>
-    <row r="81" spans="1:8">
+    <row r="81" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A81">
         <v>92</v>
       </c>
@@ -3055,7 +3070,7 @@
         <v>190</v>
       </c>
     </row>
-    <row r="82" spans="1:8">
+    <row r="82" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A82">
         <v>91</v>
       </c>
@@ -3081,7 +3096,7 @@
         <v>183</v>
       </c>
     </row>
-    <row r="83" spans="1:8">
+    <row r="83" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A83">
         <v>91</v>
       </c>
@@ -3107,7 +3122,7 @@
         <v>191</v>
       </c>
     </row>
-    <row r="84" spans="1:8">
+    <row r="84" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A84">
         <v>91</v>
       </c>
@@ -3133,7 +3148,7 @@
         <v>183</v>
       </c>
     </row>
-    <row r="85" spans="1:8">
+    <row r="85" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A85">
         <v>91</v>
       </c>
@@ -3159,7 +3174,7 @@
         <v>192</v>
       </c>
     </row>
-    <row r="86" spans="1:8">
+    <row r="86" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A86">
         <v>91</v>
       </c>
@@ -3185,7 +3200,7 @@
         <v>183</v>
       </c>
     </row>
-    <row r="87" spans="1:8">
+    <row r="87" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A87">
         <v>91</v>
       </c>
@@ -3211,7 +3226,7 @@
         <v>183</v>
       </c>
     </row>
-    <row r="88" spans="1:8">
+    <row r="88" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A88">
         <v>91</v>
       </c>
@@ -3237,7 +3252,7 @@
         <v>183</v>
       </c>
     </row>
-    <row r="89" spans="1:8">
+    <row r="89" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A89">
         <v>91</v>
       </c>
@@ -3263,7 +3278,7 @@
         <v>183</v>
       </c>
     </row>
-    <row r="90" spans="1:8">
+    <row r="90" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A90">
         <v>91</v>
       </c>
@@ -3289,7 +3304,7 @@
         <v>183</v>
       </c>
     </row>
-    <row r="91" spans="1:8">
+    <row r="91" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A91">
         <v>91</v>
       </c>
@@ -3315,7 +3330,7 @@
         <v>183</v>
       </c>
     </row>
-    <row r="92" spans="1:8">
+    <row r="92" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A92">
         <v>91</v>
       </c>
@@ -3341,7 +3356,7 @@
         <v>183</v>
       </c>
     </row>
-    <row r="93" spans="1:8">
+    <row r="93" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A93">
         <v>91</v>
       </c>
@@ -3367,7 +3382,7 @@
         <v>171</v>
       </c>
     </row>
-    <row r="94" spans="1:8">
+    <row r="94" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A94">
         <v>91</v>
       </c>
@@ -3393,7 +3408,7 @@
         <v>193</v>
       </c>
     </row>
-    <row r="95" spans="1:8">
+    <row r="95" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A95">
         <v>91</v>
       </c>
@@ -3419,7 +3434,7 @@
         <v>190</v>
       </c>
     </row>
-    <row r="96" spans="1:8">
+    <row r="96" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A96">
         <v>91</v>
       </c>
@@ -3445,7 +3460,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="97" spans="1:8">
+    <row r="97" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A97">
         <v>91</v>
       </c>
@@ -3471,7 +3486,7 @@
         <v>194</v>
       </c>
     </row>
-    <row r="98" spans="1:8">
+    <row r="98" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A98">
         <v>91</v>
       </c>
@@ -3497,7 +3512,7 @@
         <v>167</v>
       </c>
     </row>
-    <row r="99" spans="1:8">
+    <row r="99" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A99">
         <v>91</v>
       </c>
@@ -3523,7 +3538,7 @@
         <v>170</v>
       </c>
     </row>
-    <row r="100" spans="1:8">
+    <row r="100" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A100">
         <v>91</v>
       </c>
@@ -3549,7 +3564,7 @@
         <v>176</v>
       </c>
     </row>
-    <row r="101" spans="1:8">
+    <row r="101" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A101">
         <v>91</v>
       </c>
@@ -3575,7 +3590,7 @@
         <v>165</v>
       </c>
     </row>
-    <row r="102" spans="1:8">
+    <row r="102" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A102">
         <v>91</v>
       </c>
@@ -3601,7 +3616,7 @@
         <v>179</v>
       </c>
     </row>
-    <row r="103" spans="1:8">
+    <row r="103" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A103">
         <v>91</v>
       </c>
@@ -3627,7 +3642,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="104" spans="1:8">
+    <row r="104" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A104">
         <v>90</v>
       </c>
@@ -3653,7 +3668,7 @@
         <v>168</v>
       </c>
     </row>
-    <row r="105" spans="1:8">
+    <row r="105" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A105">
         <v>90</v>
       </c>
@@ -3679,7 +3694,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="106" spans="1:8">
+    <row r="106" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A106">
         <v>90</v>
       </c>

</xml_diff>